<commit_message>
Pre Market Tue 2026-06-30
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-06-30.xlsx
+++ b/market-prep/Pre Market 2026-06-30.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7440,26</t>
+          <t>7440,44</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29741,93</t>
+          <t>29774,75</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3010,40</t>
+          <t>3010,42</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>52182,07</t>
+          <t>52182,75</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4015,29</t>
+          <t>4015,47</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>58,20</t>
+          <t>58,27</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1580,30</t>
+          <t>1578,70</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>73,63</t>
+          <t>73,91</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>60388,76</t>
+          <t>60220,49</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,12 +680,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1622,33</t>
+          <t>1613,45</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6++</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-4,40%</t>
+          <t>-4,13%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7436,32</t>
+          <t>7440,43</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>